<commit_message>
Calibra category_rules.csv com os Document Type reais e corrige CNPJ
- category_rules.csv agora tem coluna_valor por tipo de documento, porque
  ZOR/ZREA carregam o valor em Value Reserved, não em Value Confirmed
  (Value Confirmed vem sempre 0 pra esses dois).
- audit() mostra soma de Value Confirmed e Value Reserved lado a lado,
  pra deixar isso óbvio sem precisar perguntar de novo.
- Corrige Root CNPJ sendo lido como número e perdendo zero à esquerda
  (dtype forçado pra string na leitura + zfill de segurança).
- category_rules.csv calibrado com ZTO/ZOR/ZF2/ZG2/ZREA confirmados.
</commit_message>
<xml_diff>
--- a/movimentacao_consolidada/sample_data/exemplo_movimentacao.xlsx
+++ b/movimentacao_consolidada/sample_data/exemplo_movimentacao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:G129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,11 @@
           <t>Value Confirmed</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Value Reserved</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -473,12 +478,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>1327.05</v>
       </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -507,6 +515,9 @@
       <c r="F3" t="n">
         <v>-40583.28</v>
       </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -529,10 +540,13 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
         <v>-37763.09</v>
       </c>
     </row>
@@ -557,10 +571,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
         <v>-42460.14</v>
       </c>
     </row>
@@ -585,10 +602,13 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
         <v>-22089.24</v>
       </c>
     </row>
@@ -609,15 +629,18 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>4362.38</v>
+        <v>6373.94</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -641,12 +664,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>-38207.31</v>
       </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -669,10 +695,13 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
         <v>-42315.63</v>
       </c>
     </row>
@@ -693,15 +722,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>73168.46000000001</v>
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-33905.75</v>
       </c>
     </row>
     <row r="11">
@@ -721,15 +753,18 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>31566.32</v>
+        <v>31981.37</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -759,6 +794,9 @@
       <c r="F12" t="n">
         <v>25023.38</v>
       </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -781,10 +819,13 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
         <v>-43553.39</v>
       </c>
     </row>
@@ -809,12 +850,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>-43944.25</v>
       </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -837,12 +881,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>-12350.79</v>
       </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -865,12 +912,15 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>20289.17</v>
       </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -889,15 +939,18 @@
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>22833.45</v>
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-9897.360000000001</v>
       </c>
     </row>
     <row r="18">
@@ -917,15 +970,18 @@
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-26505.57</v>
+        <v>-36602.76</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -945,15 +1001,18 @@
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>24256.57</v>
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>33058.75</v>
       </c>
     </row>
     <row r="20">
@@ -977,11 +1036,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>-1588.32</v>
+        <v>21206.78</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1005,11 +1067,14 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>42574.4</v>
+        <v>23367.88</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1033,11 +1098,14 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>-42251.85</v>
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-23225.37</v>
       </c>
     </row>
     <row r="23">
@@ -1061,11 +1129,14 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>14533.88</v>
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>5587</v>
       </c>
     </row>
     <row r="24">
@@ -1076,24 +1147,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>45453214</t>
+          <t>07224991</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PROFARMA DIST PROD FCEUTICO SA</t>
+          <t>NAZARIA DIST PROD FCEUTICO LTDA</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>51039.74</v>
+        <v>10528.24</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1104,24 +1178,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>45453214</t>
+          <t>07224991</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PROFARMA DIST PROD FCEUTICO SA</t>
+          <t>NAZARIA DIST PROD FCEUTICO LTDA</t>
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>26123.04</v>
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-2994.29</v>
       </c>
     </row>
     <row r="26">
@@ -1145,11 +1222,14 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>-2994.29</v>
+        <v>40869.28</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1173,11 +1253,14 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>53269.33</v>
+        <v>-39358.85</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1201,11 +1284,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>51377.85</v>
+        <v>18275.55</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1229,11 +1315,14 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>24675.08</v>
+        <v>44827.89</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1257,11 +1346,14 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>14365.13</v>
+        <v>29164.67</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1285,11 +1377,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>8348.440000000001</v>
+        <v>16551.27</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1313,11 +1408,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>77422.73</v>
+        <v>48428.32</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1341,11 +1439,14 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>16551.27</v>
+        <v>71325.13</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1369,11 +1470,14 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>48428.32</v>
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-44903.06</v>
       </c>
     </row>
     <row r="35">
@@ -1393,15 +1497,18 @@
         </is>
       </c>
       <c r="D35" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>71325.13</v>
+        <v>49394.21</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1425,11 +1532,14 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>75062.48</v>
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>52582.24</v>
       </c>
     </row>
     <row r="37">
@@ -1453,11 +1563,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>49394.21</v>
+        <v>-5784.09</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1481,11 +1594,14 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>52582.24</v>
+        <v>27268.08</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1509,11 +1625,14 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>-5784.09</v>
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>53595.96</v>
       </c>
     </row>
     <row r="40">
@@ -1537,11 +1656,14 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>27268.08</v>
+        <v>59195.81</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1565,11 +1687,14 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>53595.96</v>
+        <v>11632.78</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1589,7 +1714,7 @@
         </is>
       </c>
       <c r="D42" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1597,7 +1722,10 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>72808.53999999999</v>
+        <v>-42112.97</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1617,15 +1745,18 @@
         </is>
       </c>
       <c r="D43" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>40615.47</v>
+        <v>34126.75</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1649,11 +1780,14 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>-42112.97</v>
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-13002.58</v>
       </c>
     </row>
     <row r="45">
@@ -1664,24 +1798,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D45" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>34126.75</v>
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>65315.24</v>
       </c>
     </row>
     <row r="46">
@@ -1692,24 +1829,27 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D46" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>56850.22</v>
+        <v>-47066.82</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1720,24 +1860,27 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D47" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>43161.61</v>
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-3789.67</v>
       </c>
     </row>
     <row r="48">
@@ -1748,24 +1891,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D48" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>-4889.32</v>
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-34777.55</v>
       </c>
     </row>
     <row r="49">
@@ -1776,24 +1922,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D49" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>-3789.67</v>
+        <v>-21632.99</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -1804,24 +1953,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D50" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>-34777.55</v>
+        <v>-33185.77</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1832,24 +1984,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D51" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>-21632.99</v>
+        <v>1726.7</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1860,24 +2015,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>61940292</t>
+          <t>45453214</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>DIST MEDIC SANTA CRUZ LTDA</t>
+          <t>PROFARMA DIST PROD FCEUTICO SA</t>
         </is>
       </c>
       <c r="D52" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>-33185.77</v>
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-39524.43</v>
       </c>
     </row>
     <row r="53">
@@ -1897,15 +2055,18 @@
         </is>
       </c>
       <c r="D53" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>823.46</v>
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>21427.19</v>
       </c>
     </row>
     <row r="54">
@@ -1925,15 +2086,18 @@
         </is>
       </c>
       <c r="D54" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>-39524.43</v>
+        <v>56506.38</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1953,15 +2117,18 @@
         </is>
       </c>
       <c r="D55" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>2213.75</v>
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-13805.26</v>
       </c>
     </row>
     <row r="56">
@@ -1981,15 +2148,18 @@
         </is>
       </c>
       <c r="D56" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>64839.9</v>
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>78240.72</v>
       </c>
     </row>
     <row r="57">
@@ -2009,15 +2179,18 @@
         </is>
       </c>
       <c r="D57" s="1" t="n">
-        <v>46174</v>
+        <v>46113</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>-13805.26</v>
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>74505.06</v>
       </c>
     </row>
     <row r="58">
@@ -2037,15 +2210,18 @@
         </is>
       </c>
       <c r="D58" s="1" t="n">
-        <v>46174</v>
+        <v>46113</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>78240.72</v>
+        <v>-39211.99</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -2065,15 +2241,18 @@
         </is>
       </c>
       <c r="D59" s="1" t="n">
-        <v>46174</v>
+        <v>46113</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>64945.07</v>
+        <v>-19845.61</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2093,15 +2272,18 @@
         </is>
       </c>
       <c r="D60" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>-30380.28</v>
+        <v>13045.15</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -2121,15 +2303,18 @@
         </is>
       </c>
       <c r="D61" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>-30331.21</v>
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-26295.43</v>
       </c>
     </row>
     <row r="62">
@@ -2149,15 +2334,18 @@
         </is>
       </c>
       <c r="D62" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>-19666.31</v>
+        <v>-49467.83</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -2177,15 +2365,18 @@
         </is>
       </c>
       <c r="D63" s="1" t="n">
-        <v>46204</v>
+        <v>46143</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>-26295.43</v>
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>19496.83</v>
       </c>
     </row>
     <row r="64">
@@ -2205,15 +2396,18 @@
         </is>
       </c>
       <c r="D64" s="1" t="n">
-        <v>46204</v>
+        <v>46143</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>-49467.83</v>
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>23624.36</v>
       </c>
     </row>
     <row r="65">
@@ -2233,15 +2427,18 @@
         </is>
       </c>
       <c r="D65" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>19496.83</v>
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>73529.11</v>
       </c>
     </row>
     <row r="66">
@@ -2261,15 +2458,18 @@
         </is>
       </c>
       <c r="D66" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>23624.36</v>
+        <v>9363.68</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -2289,15 +2489,18 @@
         </is>
       </c>
       <c r="D67" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>39764.18</v>
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>1009.26</v>
       </c>
     </row>
     <row r="68">
@@ -2317,15 +2520,18 @@
         </is>
       </c>
       <c r="D68" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>73529.11</v>
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>1235.6</v>
       </c>
     </row>
     <row r="69">
@@ -2336,24 +2542,27 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>46054219</t>
+          <t>61940292</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SOLFARMA COM PROD FCEUTICO S A</t>
+          <t>DIST MEDIC SANTA CRUZ LTDA</t>
         </is>
       </c>
       <c r="D69" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>46172.02</v>
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>32457.64</v>
       </c>
     </row>
     <row r="70">
@@ -2364,24 +2573,27 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>46054219</t>
+          <t>61940292</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SOLFARMA COM PROD FCEUTICO S A</t>
+          <t>DIST MEDIC SANTA CRUZ LTDA</t>
         </is>
       </c>
       <c r="D70" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>66939.28999999999</v>
+        <v>-41244.81</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2392,24 +2604,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>46054219</t>
+          <t>61940292</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SOLFARMA COM PROD FCEUTICO S A</t>
+          <t>DIST MEDIC SANTA CRUZ LTDA</t>
         </is>
       </c>
       <c r="D71" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>53723.51</v>
+        <v>7281.49</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2420,24 +2635,27 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>46054219</t>
+          <t>61940292</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SOLFARMA COM PROD FCEUTICO S A</t>
+          <t>DIST MEDIC SANTA CRUZ LTDA</t>
         </is>
       </c>
       <c r="D72" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>1749.05</v>
+        <v>-5793.03</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -2448,24 +2666,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>46054219</t>
+          <t>61940292</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SOLFARMA COM PROD FCEUTICO S A</t>
+          <t>DIST MEDIC SANTA CRUZ LTDA</t>
         </is>
       </c>
       <c r="D73" s="1" t="n">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>-36540.18</v>
+        <v>-36690.65</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2489,11 +2710,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>2057.54</v>
+        <v>19760.43</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2517,11 +2741,14 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>-41244.81</v>
+        <v>29785.84</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -2545,11 +2772,14 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>7281.49</v>
+        <v>63663.21</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2569,15 +2799,18 @@
         </is>
       </c>
       <c r="D77" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>28094.54</v>
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-1090.18</v>
       </c>
     </row>
     <row r="78">
@@ -2597,15 +2830,18 @@
         </is>
       </c>
       <c r="D78" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>-49969.67</v>
+        <v>74210.84</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2625,15 +2861,18 @@
         </is>
       </c>
       <c r="D79" s="1" t="n">
-        <v>46143</v>
+        <v>46113</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>19760.43</v>
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-2658.75</v>
       </c>
     </row>
     <row r="80">
@@ -2653,15 +2892,18 @@
         </is>
       </c>
       <c r="D80" s="1" t="n">
-        <v>46174</v>
+        <v>46113</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>-46684.88</v>
+        <v>-35004.04</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2681,15 +2923,18 @@
         </is>
       </c>
       <c r="D81" s="1" t="n">
-        <v>46174</v>
+        <v>46113</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>29828.97</v>
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>79103.35000000001</v>
       </c>
     </row>
     <row r="82">
@@ -2709,15 +2954,18 @@
         </is>
       </c>
       <c r="D82" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>32473.25</v>
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>12898.51</v>
       </c>
     </row>
     <row r="83">
@@ -2737,15 +2985,18 @@
         </is>
       </c>
       <c r="D83" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>28296.29</v>
+        <v>-31264.73</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -2765,15 +3016,18 @@
         </is>
       </c>
       <c r="D84" s="1" t="n">
-        <v>46174</v>
+        <v>46143</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>-34030.51</v>
+        <v>46245.66</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -2793,15 +3047,18 @@
         </is>
       </c>
       <c r="D85" s="1" t="n">
-        <v>46204</v>
+        <v>46143</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>12451.36</v>
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>57751.2</v>
       </c>
     </row>
     <row r="86">
@@ -2821,15 +3078,18 @@
         </is>
       </c>
       <c r="D86" s="1" t="n">
-        <v>46204</v>
+        <v>46143</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>-38834.99</v>
+        <v>17123.49</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -2849,15 +3109,18 @@
         </is>
       </c>
       <c r="D87" s="1" t="n">
-        <v>46204</v>
+        <v>46143</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>47457.61</v>
+        <v>73628.12</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -2877,15 +3140,18 @@
         </is>
       </c>
       <c r="D88" s="1" t="n">
-        <v>46204</v>
+        <v>46143</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>-15581.6</v>
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
+        <v>-2972.18</v>
       </c>
     </row>
     <row r="89">
@@ -2905,15 +3171,18 @@
         </is>
       </c>
       <c r="D89" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>-29012.98</v>
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
+        <v>68838.95</v>
       </c>
     </row>
     <row r="90">
@@ -2933,15 +3202,18 @@
         </is>
       </c>
       <c r="D90" s="1" t="n">
-        <v>46204</v>
+        <v>46174</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>-23322.05</v>
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>-11248.34</v>
       </c>
     </row>
     <row r="91">
@@ -2952,24 +3224,27 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D91" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>-30941.67</v>
+        <v>40505.58</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -2980,24 +3255,27 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D92" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>68838.95</v>
+        <v>17391.59</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -3008,24 +3286,27 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D93" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>-11248.34</v>
+        <v>-3759.5</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -3036,24 +3317,27 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D94" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>62232.25</v>
+        <v>19237.01</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -3064,24 +3348,27 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D95" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>59908.19</v>
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
+        <v>-7143.55</v>
       </c>
     </row>
     <row r="96">
@@ -3092,24 +3379,27 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D96" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>-2329.03</v>
+        <v>29719.67</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -3120,24 +3410,27 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D97" s="1" t="n">
-        <v>46113</v>
+        <v>46174</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>-3759.5</v>
+        <v>54790.22</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -3148,24 +3441,27 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D98" s="1" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>20403.73</v>
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
+        <v>46183.49</v>
       </c>
     </row>
     <row r="99">
@@ -3176,24 +3472,27 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D99" s="1" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ZOF</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>-7143.55</v>
+        <v>-24010.66</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -3204,24 +3503,27 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D100" s="1" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>29719.67</v>
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
+        <v>-3776.87</v>
       </c>
     </row>
     <row r="101">
@@ -3232,24 +3534,27 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D101" s="1" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>54790.22</v>
+        <v>78648.47</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -3260,24 +3565,27 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D102" s="1" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>54432.39</v>
+        <v>11391.21</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -3288,24 +3596,27 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D103" s="1" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>ZRE</t>
+          <t>ZF2</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>17293.03</v>
+        <v>40027.85</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -3316,24 +3627,27 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D104" s="1" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>45030.52</v>
+        <v>8139.6</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -3344,24 +3658,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D105" s="1" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>52714.84</v>
+        <v>74150.08</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -3372,24 +3689,27 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D106" s="1" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>-16307.33</v>
+        <v>-39530.04</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -3400,24 +3720,27 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>39455032</t>
+          <t>46054219</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>MEDNORTE DIST MEDIC LTDA</t>
+          <t>SOLFARMA COM PROD FCEUTICO S A</t>
         </is>
       </c>
       <c r="D107" s="1" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZTO</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>28668.07</v>
+        <v>-20510.04</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -3437,15 +3760,18 @@
         </is>
       </c>
       <c r="D108" s="1" t="n">
-        <v>46204</v>
+        <v>46113</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>ZRC</t>
+          <t>ZG2</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>55113.55</v>
+        <v>-23431.46</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -3465,15 +3791,18 @@
         </is>
       </c>
       <c r="D109" s="1" t="n">
-        <v>46204</v>
+        <v>46113</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>ZFT</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>78444.95</v>
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
+        <v>78082.37</v>
       </c>
     </row>
     <row r="110">
@@ -3493,15 +3822,18 @@
         </is>
       </c>
       <c r="D110" s="1" t="n">
-        <v>46204</v>
+        <v>46113</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>ZCA</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>-39530.04</v>
+        <v>0</v>
+      </c>
+      <c r="G110" t="n">
+        <v>59256.62</v>
       </c>
     </row>
     <row r="111">
@@ -3521,15 +3853,18 @@
         </is>
       </c>
       <c r="D111" s="1" t="n">
-        <v>46204</v>
+        <v>46113</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>-20510.04</v>
+        <v>0</v>
+      </c>
+      <c r="G111" t="n">
+        <v>68195.89999999999</v>
       </c>
     </row>
     <row r="112">
@@ -3549,15 +3884,545 @@
         </is>
       </c>
       <c r="D112" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>ZG2</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>53953.69</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ZTO</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>68271.03</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>12144.26</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D115" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>6410.26</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D116" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>ZG2</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>-38722.52</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D117" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>ZOR</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>10210.87</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D118" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>ZTO</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>44223.83</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D119" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>79104.61</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ZTO</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>-30350.41</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>ZOR</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" t="n">
+        <v>54845.26</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D122" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>29504.53</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D123" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ZREA</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="n">
+        <v>77439.77</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D124" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>ZG2</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>-29731.38</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>ZREA</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" t="n">
+        <v>-32972.1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D126" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>ZRE</t>
-        </is>
-      </c>
-      <c r="F112" t="n">
-        <v>-6094.13</v>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>ZTO</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>18455.54</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D127" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>6395.23</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D128" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>57400.18</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>X401</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>39455032</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>MEDNORTE DIST MEDIC LTDA</t>
+        </is>
+      </c>
+      <c r="D129" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>ZF2</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>-46360.82</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reestrutura em painéis por abas separadas + aba de Notas Fiscais
- Painel Cliente Faturado (Ressarcimento SAP + Faturado em Nota + ajustes)
  e Painel Cliente Reservado (Ressarcimento SAP + Reserva + ajustes) viram
  abas independentes (não mais blocos lado a lado), cada uma com sua
  própria fórmula/tabela de origem.
- Geral e Por Cliente passam a mostrar só o painel principal (Faturado);
  Por Cliente ganha uma tabela auxiliar pro painel Reservado.
- Nova aba Notas Fiscais: detalhe por nota (Mês, Nome Cliente, CNPJ, NFE
  Number, NFE Item, PO Number, Value Confirmed) pra ZS1/ZS2/ZF1/ZF2,
  direto do bruto, sem passar por category_rules.csv.
- category_rules.csv ganha a categoria especial "(fora do waterfall)"
  pra Document Type que só interessam na aba de Notas Fiscais.
</commit_message>
<xml_diff>
--- a/movimentacao_consolidada/sample_data/exemplo_movimentacao.xlsx
+++ b/movimentacao_consolidada/sample_data/exemplo_movimentacao.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G129"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,21 @@
           <t>Value Reserved</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>NFE Number</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>NFE Item</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PO Number</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,6 +502,21 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NF1001</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>PO1001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -518,6 +548,21 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NF1002</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PO1002</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -540,14 +585,29 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>-37763.09</v>
       </c>
       <c r="G4" t="n">
-        <v>-37763.09</v>
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NF1003</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PO1003</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -571,14 +631,29 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>-42460.14</v>
       </c>
       <c r="G5" t="n">
-        <v>-42460.14</v>
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NF1004</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PO1004</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -602,14 +677,29 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>-22089.24</v>
       </c>
       <c r="G6" t="n">
-        <v>-22089.24</v>
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NF1005</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PO1005</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -633,7 +723,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -642,6 +732,21 @@
       <c r="G7" t="n">
         <v>0</v>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NF1006</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>PO1006</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -664,7 +769,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -673,6 +778,21 @@
       <c r="G8" t="n">
         <v>0</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NF1007</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PO1007</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -695,7 +815,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -704,6 +824,21 @@
       <c r="G9" t="n">
         <v>-42315.63</v>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NF1008</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>PO1008</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -726,14 +861,29 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>-33905.75</v>
       </c>
       <c r="G10" t="n">
-        <v>-33905.75</v>
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NF1009</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>PO1009</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -757,7 +907,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -766,6 +916,21 @@
       <c r="G11" t="n">
         <v>0</v>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NF1010</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>PO1010</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -797,6 +962,21 @@
       <c r="G12" t="n">
         <v>0</v>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NF1011</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>PO1011</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -819,7 +999,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -828,6 +1008,21 @@
       <c r="G13" t="n">
         <v>-43553.39</v>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NF1012</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>PO1012</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -850,7 +1045,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -859,6 +1054,21 @@
       <c r="G14" t="n">
         <v>0</v>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NF1013</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>PO1013</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -890,6 +1100,21 @@
       <c r="G15" t="n">
         <v>0</v>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NF1014</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>PO1014</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -921,6 +1146,21 @@
       <c r="G16" t="n">
         <v>0</v>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NF1015</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>PO1015</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -943,14 +1183,29 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>-9897.360000000001</v>
       </c>
       <c r="G17" t="n">
-        <v>-9897.360000000001</v>
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NF1016</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PO1016</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -983,6 +1238,21 @@
       <c r="G18" t="n">
         <v>0</v>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NF1017</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>PO1017</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1005,14 +1275,29 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>33058.75</v>
       </c>
       <c r="G19" t="n">
-        <v>33058.75</v>
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>NF1018</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>PO1018</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1036,7 +1321,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1045,6 +1330,21 @@
       <c r="G20" t="n">
         <v>0</v>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NF1019</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>PO1019</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1067,7 +1367,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1076,6 +1376,21 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NF1020</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>PO1020</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1098,14 +1413,29 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>-23225.37</v>
       </c>
       <c r="G22" t="n">
-        <v>-23225.37</v>
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NF1021</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>PO1021</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1129,14 +1459,29 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>5587</v>
       </c>
       <c r="G23" t="n">
-        <v>5587</v>
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NF1022</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>PO1022</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1160,14 +1505,29 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
         <v>10528.24</v>
       </c>
-      <c r="G24" t="n">
-        <v>0</v>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NF1023</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>PO1023</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1191,7 +1551,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1200,6 +1560,21 @@
       <c r="G25" t="n">
         <v>-2994.29</v>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NF1024</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>PO1024</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1231,6 +1606,21 @@
       <c r="G26" t="n">
         <v>0</v>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NF1025</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>PO1025</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1253,7 +1643,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1262,6 +1652,21 @@
       <c r="G27" t="n">
         <v>0</v>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>NF1026</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>PO1026</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1293,6 +1698,21 @@
       <c r="G28" t="n">
         <v>0</v>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>NF1027</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>PO1027</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1315,14 +1735,29 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
         <v>44827.89</v>
       </c>
-      <c r="G29" t="n">
-        <v>0</v>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NF1028</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>PO1028</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1355,6 +1790,21 @@
       <c r="G30" t="n">
         <v>0</v>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>NF1029</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>PO1029</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1377,7 +1827,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1386,6 +1836,21 @@
       <c r="G31" t="n">
         <v>0</v>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NF1030</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>PO1030</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1417,6 +1882,21 @@
       <c r="G32" t="n">
         <v>0</v>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>NF1031</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>PO1031</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1448,6 +1928,21 @@
       <c r="G33" t="n">
         <v>0</v>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NF1032</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>PO1032</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1470,7 +1965,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1479,6 +1974,21 @@
       <c r="G34" t="n">
         <v>-44903.06</v>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>NF1033</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>PO1033</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1501,7 +2011,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1510,6 +2020,21 @@
       <c r="G35" t="n">
         <v>0</v>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NF1034</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>PO1034</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1532,14 +2057,29 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>52582.24</v>
       </c>
       <c r="G36" t="n">
-        <v>52582.24</v>
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NF1035</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>PO1035</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1563,14 +2103,29 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
         <v>-5784.09</v>
       </c>
-      <c r="G37" t="n">
-        <v>0</v>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NF1036</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>PO1036</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1594,14 +2149,29 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
         <v>27268.08</v>
       </c>
-      <c r="G38" t="n">
-        <v>0</v>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NF1037</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>PO1037</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1625,14 +2195,29 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>53595.96</v>
       </c>
       <c r="G39" t="n">
-        <v>53595.96</v>
+        <v>0</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NF1038</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>PO1038</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1656,7 +2241,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1665,6 +2250,21 @@
       <c r="G40" t="n">
         <v>0</v>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>NF1039</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>PO1039</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1696,6 +2296,21 @@
       <c r="G41" t="n">
         <v>0</v>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NF1040</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>PO1040</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1718,7 +2333,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -1727,6 +2342,21 @@
       <c r="G42" t="n">
         <v>0</v>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NF1041</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>PO1041</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1758,6 +2388,21 @@
       <c r="G43" t="n">
         <v>0</v>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NF1042</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>PO1042</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1780,7 +2425,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -1789,6 +2434,21 @@
       <c r="G44" t="n">
         <v>-13002.58</v>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>NF1043</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PO1043</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1811,7 +2471,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -1820,6 +2480,21 @@
       <c r="G45" t="n">
         <v>65315.24</v>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NF1044</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>PO1044</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1842,14 +2517,29 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
         <v>-47066.82</v>
       </c>
-      <c r="G46" t="n">
-        <v>0</v>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>NF1045</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>PO1045</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1873,7 +2563,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -1882,6 +2572,21 @@
       <c r="G47" t="n">
         <v>-3789.67</v>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>NF1046</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>PO1046</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1904,14 +2609,29 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>-34777.55</v>
       </c>
       <c r="G48" t="n">
-        <v>-34777.55</v>
+        <v>0</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>NF1047</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>PO1047</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -1944,6 +2664,21 @@
       <c r="G49" t="n">
         <v>0</v>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>NF1048</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>PO1048</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1975,6 +2710,21 @@
       <c r="G50" t="n">
         <v>0</v>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>NF1049</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>PO1049</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1997,7 +2747,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -2006,6 +2756,21 @@
       <c r="G51" t="n">
         <v>0</v>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>NF1050</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>PO1050</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2028,7 +2793,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -2037,6 +2802,21 @@
       <c r="G52" t="n">
         <v>-39524.43</v>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>NF1051</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>PO1051</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2059,7 +2839,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2068,6 +2848,21 @@
       <c r="G53" t="n">
         <v>21427.19</v>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>NF1052</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>PO1052</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2099,6 +2894,21 @@
       <c r="G54" t="n">
         <v>0</v>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>NF1053</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>PO1053</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2121,14 +2931,29 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>-13805.26</v>
       </c>
       <c r="G55" t="n">
-        <v>-13805.26</v>
+        <v>0</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>NF1054</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>PO1054</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -2152,7 +2977,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -2161,6 +2986,21 @@
       <c r="G56" t="n">
         <v>78240.72</v>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>NF1055</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>PO1055</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2183,7 +3023,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2192,6 +3032,21 @@
       <c r="G57" t="n">
         <v>74505.06</v>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>NF1056</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>PO1056</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2223,6 +3078,21 @@
       <c r="G58" t="n">
         <v>0</v>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>NF1057</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>PO1057</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2254,6 +3124,21 @@
       <c r="G59" t="n">
         <v>0</v>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>NF1058</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>PO1058</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2285,6 +3170,21 @@
       <c r="G60" t="n">
         <v>0</v>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>NF1059</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PO1059</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2307,14 +3207,29 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
+        <v>-26295.43</v>
       </c>
       <c r="G61" t="n">
-        <v>-26295.43</v>
+        <v>0</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>NF1060</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>PO1060</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -2347,6 +3262,21 @@
       <c r="G62" t="n">
         <v>0</v>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>NF1061</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>PO1061</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2369,7 +3299,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -2378,6 +3308,21 @@
       <c r="G63" t="n">
         <v>19496.83</v>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>NF1062</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PO1062</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2400,14 +3345,29 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
+        <v>23624.36</v>
       </c>
       <c r="G64" t="n">
-        <v>23624.36</v>
+        <v>0</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>NF1063</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>PO1063</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -2431,14 +3391,29 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>73529.11</v>
       </c>
       <c r="G65" t="n">
-        <v>73529.11</v>
+        <v>0</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>NF1064</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>PO1064</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -2471,6 +3446,21 @@
       <c r="G66" t="n">
         <v>0</v>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>NF1065</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PO1065</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2493,14 +3483,29 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0</v>
+        <v>1009.26</v>
       </c>
       <c r="G67" t="n">
-        <v>1009.26</v>
+        <v>0</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>NF1066</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>PO1066</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -2524,7 +3529,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -2533,6 +3538,21 @@
       <c r="G68" t="n">
         <v>1235.6</v>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>NF1067</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>PO1067</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2555,7 +3575,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -2564,6 +3584,21 @@
       <c r="G69" t="n">
         <v>32457.64</v>
       </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>NF1068</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>PO1068</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2586,7 +3621,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -2595,6 +3630,21 @@
       <c r="G70" t="n">
         <v>0</v>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>NF1069</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>PO1069</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2617,7 +3667,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -2626,6 +3676,21 @@
       <c r="G71" t="n">
         <v>0</v>
       </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>NF1070</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>PO1070</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2648,7 +3713,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -2657,6 +3722,21 @@
       <c r="G72" t="n">
         <v>0</v>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>NF1071</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>PO1071</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2688,6 +3768,21 @@
       <c r="G73" t="n">
         <v>0</v>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>NF1072</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>PO1072</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2719,6 +3814,21 @@
       <c r="G74" t="n">
         <v>0</v>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>NF1073</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>PO1073</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2741,14 +3851,29 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
         <v>29785.84</v>
       </c>
-      <c r="G75" t="n">
-        <v>0</v>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>NF1074</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>PO1074</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -2772,7 +3897,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -2781,6 +3906,21 @@
       <c r="G76" t="n">
         <v>0</v>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>NF1075</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>PO1075</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2803,14 +3943,29 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>-1090.18</v>
       </c>
       <c r="G77" t="n">
-        <v>-1090.18</v>
+        <v>0</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>NF1076</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>PO1076</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -2843,6 +3998,21 @@
       <c r="G78" t="n">
         <v>0</v>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>NF1077</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>PO1077</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2865,14 +4035,29 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0</v>
+        <v>-2658.75</v>
       </c>
       <c r="G79" t="n">
-        <v>-2658.75</v>
+        <v>0</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>NF1078</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>PO1078</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -2896,7 +4081,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -2905,6 +4090,21 @@
       <c r="G80" t="n">
         <v>0</v>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>NF1079</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>PO1079</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2927,7 +4127,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -2936,6 +4136,21 @@
       <c r="G81" t="n">
         <v>79103.35000000001</v>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>NF1080</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>PO1080</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2958,7 +4173,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -2967,6 +4182,21 @@
       <c r="G82" t="n">
         <v>12898.51</v>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>NF1081</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>PO1081</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2989,7 +4219,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -2998,6 +4228,21 @@
       <c r="G83" t="n">
         <v>0</v>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>NF1082</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>PO1082</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3020,14 +4265,29 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
         <v>46245.66</v>
       </c>
-      <c r="G84" t="n">
-        <v>0</v>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>NF1083</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>PO1083</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -3051,7 +4311,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -3060,6 +4320,21 @@
       <c r="G85" t="n">
         <v>57751.2</v>
       </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>NF1084</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>PO1084</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3091,6 +4366,21 @@
       <c r="G86" t="n">
         <v>0</v>
       </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>NF1085</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>PO1085</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3113,7 +4403,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -3122,6 +4412,21 @@
       <c r="G87" t="n">
         <v>0</v>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>NF1086</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>PO1086</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3144,14 +4449,29 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>-2972.18</v>
       </c>
       <c r="G88" t="n">
-        <v>-2972.18</v>
+        <v>0</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>NF1087</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>PO1087</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -3175,14 +4495,29 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>0</v>
+        <v>68838.95</v>
       </c>
       <c r="G89" t="n">
-        <v>68838.95</v>
+        <v>0</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>NF1088</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>PO1088</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -3206,14 +4541,29 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>-11248.34</v>
       </c>
       <c r="G90" t="n">
-        <v>-11248.34</v>
+        <v>0</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>NF1089</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>PO1089</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -3237,7 +4587,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -3246,6 +4596,21 @@
       <c r="G91" t="n">
         <v>0</v>
       </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>NF1090</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>PO1090</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3277,6 +4642,21 @@
       <c r="G92" t="n">
         <v>0</v>
       </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>NF1091</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>PO1091</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3308,6 +4688,21 @@
       <c r="G93" t="n">
         <v>0</v>
       </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>NF1092</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>PO1092</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3330,7 +4725,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -3339,6 +4734,21 @@
       <c r="G94" t="n">
         <v>0</v>
       </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>NF1093</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>PO1093</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3361,14 +4771,29 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
+        <v>-7143.55</v>
       </c>
       <c r="G95" t="n">
-        <v>-7143.55</v>
+        <v>0</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>NF1094</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>PO1094</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -3392,7 +4817,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -3401,6 +4826,21 @@
       <c r="G96" t="n">
         <v>0</v>
       </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>NF1095</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>PO1095</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3423,7 +4863,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -3432,6 +4872,21 @@
       <c r="G97" t="n">
         <v>0</v>
       </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>NF1096</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>PO1096</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3454,7 +4909,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -3463,6 +4918,21 @@
       <c r="G98" t="n">
         <v>46183.49</v>
       </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>NF1097</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>PO1097</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3485,7 +4955,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -3494,6 +4964,21 @@
       <c r="G99" t="n">
         <v>0</v>
       </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>NF1098</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>PO1098</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3516,7 +5001,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -3525,6 +5010,21 @@
       <c r="G100" t="n">
         <v>-3776.87</v>
       </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>NF1099</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>PO1099</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3556,6 +5056,21 @@
       <c r="G101" t="n">
         <v>0</v>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>NF1100</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>PO1100</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3587,6 +5102,21 @@
       <c r="G102" t="n">
         <v>0</v>
       </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>NF1101</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>PO1101</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3609,7 +5139,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -3618,6 +5148,21 @@
       <c r="G103" t="n">
         <v>0</v>
       </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>NF1102</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>PO1102</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3640,14 +5185,29 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="n">
         <v>8139.6</v>
       </c>
-      <c r="G104" t="n">
-        <v>0</v>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>NF1103</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>PO1103</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -3671,14 +5231,29 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="n">
         <v>74150.08</v>
       </c>
-      <c r="G105" t="n">
-        <v>0</v>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>NF1104</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>PO1104</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -3702,14 +5277,29 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="n">
         <v>-39530.04</v>
       </c>
-      <c r="G106" t="n">
-        <v>0</v>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>NF1105</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>PO1105</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -3733,7 +5323,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -3742,6 +5332,21 @@
       <c r="G107" t="n">
         <v>0</v>
       </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>NF1106</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>PO1106</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3764,14 +5369,29 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
         <v>-23431.46</v>
       </c>
-      <c r="G108" t="n">
-        <v>0</v>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>NF1107</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>PO1107</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -3795,14 +5415,29 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>0</v>
+        <v>78082.37</v>
       </c>
       <c r="G109" t="n">
-        <v>78082.37</v>
+        <v>0</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>NF1108</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>PO1108</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -3826,14 +5461,29 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>0</v>
+        <v>59256.62</v>
       </c>
       <c r="G110" t="n">
-        <v>59256.62</v>
+        <v>0</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>NF1109</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>PO1109</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -3857,7 +5507,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -3866,6 +5516,21 @@
       <c r="G111" t="n">
         <v>68195.89999999999</v>
       </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>NF1110</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>PO1110</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3888,14 +5553,29 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="n">
         <v>53953.69</v>
       </c>
-      <c r="G112" t="n">
-        <v>0</v>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>NF1111</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>PO1111</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -3919,7 +5599,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F113" t="n">
@@ -3928,6 +5608,21 @@
       <c r="G113" t="n">
         <v>0</v>
       </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>NF1112</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>PO1112</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3950,7 +5645,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -3959,6 +5654,21 @@
       <c r="G114" t="n">
         <v>0</v>
       </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>NF1113</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>PO1113</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3990,6 +5700,21 @@
       <c r="G115" t="n">
         <v>0</v>
       </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>NF1114</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>PO1114</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4012,14 +5737,29 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
         <v>-38722.52</v>
       </c>
-      <c r="G116" t="n">
-        <v>0</v>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>NF1115</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>PO1115</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -4043,7 +5783,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREA</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -4052,6 +5792,21 @@
       <c r="G117" t="n">
         <v>10210.87</v>
       </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>NF1116</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>PO1116</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4074,7 +5829,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -4083,6 +5838,21 @@
       <c r="G118" t="n">
         <v>0</v>
       </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>NF1117</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>PO1117</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4114,6 +5884,21 @@
       <c r="G119" t="n">
         <v>0</v>
       </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>NF1118</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>PO1118</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4145,6 +5930,21 @@
       <c r="G120" t="n">
         <v>0</v>
       </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>NF1119</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>PO1119</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4167,7 +5967,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>ZOR</t>
+          <t>ZREB</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -4176,6 +5976,21 @@
       <c r="G121" t="n">
         <v>54845.26</v>
       </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>NF1120</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>PO1120</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4207,6 +6022,21 @@
       <c r="G122" t="n">
         <v>0</v>
       </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>NF1121</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>PO1121</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4229,14 +6059,29 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS2</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>0</v>
+        <v>77439.77</v>
       </c>
       <c r="G123" t="n">
-        <v>77439.77</v>
+        <v>0</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>NF1122</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>PO1122</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -4260,14 +6105,29 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>ZG2</t>
+          <t>ZOR</t>
         </is>
       </c>
       <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="n">
         <v>-29731.38</v>
       </c>
-      <c r="G124" t="n">
-        <v>0</v>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>NF1123</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>PO1123</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -4291,14 +6151,29 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>ZREA</t>
+          <t>ZS1</t>
         </is>
       </c>
       <c r="F125" t="n">
-        <v>0</v>
+        <v>-32972.1</v>
       </c>
       <c r="G125" t="n">
-        <v>-32972.1</v>
+        <v>0</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>NF1124</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>PO1124</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -4322,7 +6197,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>ZTO</t>
+          <t>ZF1</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -4331,6 +6206,21 @@
       <c r="G126" t="n">
         <v>0</v>
       </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>NF1125</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>PO1125</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4362,6 +6252,21 @@
       <c r="G127" t="n">
         <v>0</v>
       </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>NF1126</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>PO1126</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4384,7 +6289,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -4393,6 +6298,21 @@
       <c r="G128" t="n">
         <v>0</v>
       </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>NF1127</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>PO1127</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4415,7 +6335,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>ZF2</t>
+          <t>ZG1</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -4423,6 +6343,21 @@
       </c>
       <c r="G129" t="n">
         <v>0</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>NF1128</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>000010</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>PO1128</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>